<commit_message>
provato propt alternativo del baseline
</commit_message>
<xml_diff>
--- a/FISCAL/Fiscal_LDC/Classified_Fiscal_Events_Top5Percent.xlsx
+++ b/FISCAL/Fiscal_LDC/Classified_Fiscal_Events_Top5Percent.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzodelcol/Desktop/GIT/RA_4_Caggiano/FISCAL/Fiscal_LDC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D12EEE-0B58-234B-A3A9-737E9DABDDB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DECA611-1D79-1140-82BC-1908DBCBC7B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4400" yWindow="-21600" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4400" yWindow="-21600" windowWidth="16360" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="99">
   <si>
     <t>date</t>
   </si>
@@ -55,7 +55,7 @@
     <t>1961-03-27</t>
   </si>
   <si>
-    <t>In early March 1961, the Kennedy administration initiated new government spending programs. On March 1, 1961, President Kennedy established the Peace Corps by executive order, a new federal program involving foreign aid and social initiatives. Additionally, on March 24, 1961, Kennedy sent a message to Congress proposing increased federal aid for health needs, signaling an intent to expand government spending in social programs. These actions and proposals indicate a primary focus on Government Spending (G) during this period.</t>
+    <t>The House of Representatives approved the Area Redevelopment Act (H.R. 4569) on March 28, 1961, authorizing significant federal funds for loans and grants to economically distressed areas. This legislative action represents a direct increase in government spending.</t>
   </si>
   <si>
     <t>1976-11-15</t>
@@ -64,127 +64,64 @@
     <t>N</t>
   </si>
   <si>
-    <t>The date falls shortly after the 1976 presidential election. News around this time focused on the incoming Carter administration's economic agenda. President-elect Carter's team was actively formulating a significant economic stimulus package to address high unemployment and slow growth. This package, which would be formally proposed in early 1977, was widely anticipated to include both substantial tax cuts (T) and increased government spending on public works and job creation programs (G). As such, the fiscal policy news on November 15, 1976, was primarily related to the discussion and formulation of a comprehensive stimulus plan that encompassed both G and T elements, making it difficult to classify one as the sole or primary driver of news.</t>
-  </si>
-  <si>
     <t>1980-11-06</t>
   </si>
   <si>
-    <t>The date 1980-11-06 falls two days after Ronald Reagan's landslide victory in the 1980 US Presidential Election. Reagan's campaign platform heavily emphasized supply-side economics, with a central promise of significant tax cuts for individuals and businesses. While his agenda also included increased defense spending (G), the immediate and most prominent fiscal policy news and market expectations following his election were centered on the anticipated implementation of these large-scale tax reductions, which would later materialize as the Economic Recovery Tax Act of 1981 (ERTA). Thus, the news on this date primarily signaled future tax changes.</t>
-  </si>
-  <si>
     <t>1981-02-18</t>
   </si>
   <si>
-    <t>On February 18, 1981, President Reagan delivered his 'Program for Economic Recovery' speech, outlining a comprehensive fiscal plan. This plan proposed significant cuts to non-defense government spending and increases in defense spending (G), alongside substantial across-the-board individual income tax cuts (T). As both government spending and tax changes were central and substantial components of this proposed package, it is not primarily classifiable as G or T.</t>
-  </si>
-  <si>
     <t>1993-02-15</t>
   </si>
   <si>
-    <t>On February 17, 1993, President Clinton unveiled a comprehensive economic plan that included both significant spending cuts (G) and tax increases (T) aimed at deficit reduction. News on February 15th would have been in anticipation of this balanced package, which did not primarily emphasize one over the other, making it difficult to classify a single dominant driver.</t>
-  </si>
-  <si>
     <t>1993-08-09</t>
   </si>
   <si>
-    <t>On August 10, 1993, President Clinton signed the Omnibus Budget Reconciliation Act of 1993 into law. This landmark legislation, which was the subject of intense debate and news coverage around August 9th, was primarily focused on deficit reduction through significant tax increases, including raising the top individual income tax rate and corporate tax rate, and increasing the gasoline tax. While it also contained some spending cuts, the dominant fiscal policy news and impact were related to changes in taxation.</t>
-  </si>
-  <si>
     <t>1995-10-20</t>
   </si>
   <si>
-    <t>On October 20, 1995, the US government was in the midst of intense budget negotiations between the Republican-controlled Congress and President Bill Clinton, which would soon lead to government shutdowns. The primary focus of these negotiations was on federal spending levels, particularly proposed cuts to programs like Medicare and Medicaid, and the overall appropriations bills needed to fund government operations. President Clinton vetoed several appropriations bills around this time, signaling a direct conflict over government spending.</t>
-  </si>
-  <si>
     <t>1995-11-20</t>
   </si>
   <si>
-    <t>The date 1995-11-20 falls within the second federal government shutdown (November 14, 1995, to January 6, 1996). This shutdown was a direct result of an impasse between the Republican-controlled Congress and President Bill Clinton over the federal budget, primarily concerning proposed cuts to government spending, particularly social programs like Medicare and Medicaid, and the overall level of appropriations. The news was dominated by the inability to pass spending bills, directly impacting government operations and future spending levels.</t>
-  </si>
-  <si>
     <t>1997-09-03</t>
   </si>
   <si>
-    <t>The date 1997-09-03 falls shortly after the signing of the Balanced Budget Act of 1997 (August 5, 1997). This landmark legislation was a comprehensive fiscal package designed to achieve a balanced budget, incorporating significant changes to both government spending (G) and taxation (T). Key G components included reductions in Medicare and Medicaid spending, while key T components included the Child Tax Credit, education tax credits, and capital gains tax cuts. Due to its balanced nature with substantial and intertwined provisions affecting both spending and revenue, it is not clearly primarily related to either G or T.</t>
-  </si>
-  <si>
     <t>2000-01-26</t>
   </si>
   <si>
-    <t>On January 27, 2000, President Clinton delivered his State of the Union address, outlining his budget proposals for the upcoming fiscal year. These proposals, which would have been heavily anticipated and discussed on January 26, emphasized using the projected budget surplus for targeted increases in government spending on social programs such as Medicare, education, and prescription drug benefits, alongside debt reduction. While some minor tax proposals might have been included, the primary fiscal policy news from the administration focused on allocating the surplus towards specific spending initiatives.</t>
-  </si>
-  <si>
     <t>2001-01-26</t>
   </si>
   <si>
-    <t>On January 20, 2001, George W. Bush was inaugurated as President. Immediately following his inauguration, his administration's primary fiscal policy focus was the proposal of a large tax cut package. By January 26, 2001, news and discussions surrounding these proposed tax changes, which would later materialize as the Economic Growth and Tax Relief Reconciliation Act of 2001 (EGTRRA), were a dominant feature of the macroeconomic landscape.</t>
-  </si>
-  <si>
     <t>2001-09-12</t>
   </si>
   <si>
-    <t>The date 2001-09-12 is one day after the September 11th attacks. The immediate fiscal policy response was a significant increase in government spending related to national security, defense (e.g., the War on Terror), emergency relief efforts, and homeland security infrastructure, rather than primary changes to tax policy.</t>
-  </si>
-  <si>
     <t>2001-10-01</t>
   </si>
   <si>
-    <t>The period immediately following the September 11th attacks saw a significant surge in government spending related to national security, military operations (e.g., the War in Afghanistan beginning in October 2001), and emergency response and recovery efforts. This represented a substantial increase in government outlays (G).</t>
-  </si>
-  <si>
     <t>2002-01-24</t>
   </si>
   <si>
-    <t>On January 24, 2002, news reports were heavily focused on President Bush's upcoming State of the Union address (January 29) and the anticipated budget proposals for FY2003. These proposals were expected to include significant increases in defense and homeland security spending in response to the September 11th attacks, clearly indicating a primary driver of Government Spending (G).</t>
-  </si>
-  <si>
     <t>2002-05-13</t>
   </si>
   <si>
-    <t>In May 2002, the United States was heavily engaged in the War on Terror following the 9/11 attacks. This period was characterized by significant increases in government spending on defense and homeland security. While discussions around tax policy (such as making the 2001 tax cuts permanent) were present, the primary and most impactful fiscal policy news and actions were centered on the substantial increases in government outlays for national security, military operations, and the ongoing efforts to establish and fund the Department of Homeland Security.</t>
-  </si>
-  <si>
     <t>2002-12-09</t>
   </si>
   <si>
-    <t>On December 9, 2002, news reports were heavily focused on President George W. Bush's upcoming economic stimulus proposals, which were widely anticipated to include significant tax cuts aimed at boosting the economy. This indicates a primary focus on revenue-side fiscal policy changes.</t>
-  </si>
-  <si>
     <t>2003-01-06</t>
   </si>
   <si>
-    <t>On January 7, 2003, President George W. Bush proposed a significant economic stimulus package, estimated at $674 billion over 10 years. The core of this proposal was a series of tax cuts, most notably the elimination of taxes on corporate dividends and the acceleration of previously enacted income tax rate reductions. This announcement constituted major fiscal policy news primarily related to tax changes.</t>
-  </si>
-  <si>
     <t>2003-02-03</t>
   </si>
   <si>
-    <t>In early February 2003, fiscal policy news was dominated by President George W. Bush's proposed 'Jobs and Growth' plan, unveiled in January. This plan was a significant tax-cut package, including accelerating the 2001 tax cuts and eliminating taxes on corporate dividends, which was actively being debated and discussed as a major economic stimulus.</t>
-  </si>
-  <si>
     <t>2003-07-16</t>
   </si>
   <si>
-    <t>The Jobs and Growth Tax Relief Reconciliation Act of 2003 (JGTRRA), a significant tax cut package, was signed into law on May 28, 2003. On July 16, 2003, the economic impact, implementation details, and ongoing political discussions surrounding this recently enacted legislation, which reduced taxes on dividends and capital gains and accelerated other tax cuts, would have been a primary focus of fiscal policy news. While military spending for the Iraq War was ongoing, the JGTRRA represented a distinct and recent legislative change directly impacting tax revenue and economic stimulus.</t>
-  </si>
-  <si>
     <t>2003-08-26</t>
   </si>
   <si>
-    <t>The Job and Growth Tax Relief Reconciliation Act of 2003 (JGTRRA), a significant tax cut package, was signed into law in May 2003. Its economic effects, implementation, and ongoing policy discussions would still be a dominant fiscal policy 'news' item and economic driver in August 2003, representing a clear change in revenue policy.</t>
-  </si>
-  <si>
     <t>2003-08-27</t>
   </si>
   <si>
-    <t>The Jobs and Growth Tax Relief Reconciliation Act of 2003 (JGTRRA), signed into law in May 2003, significantly reduced taxes on dividends and capital gains. In August 2003, the economic effects and budget implications of these recent, substantial tax cuts were a prominent topic of fiscal policy discussion and news, making tax changes a primary driver.</t>
-  </si>
-  <si>
     <t>2004-10-07</t>
-  </si>
-  <si>
-    <t>Max Retries Reached</t>
   </si>
   <si>
     <t>2004-11-04</t>
@@ -401,24 +338,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -448,21 +373,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -769,11 +686,11 @@
   <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="108.1640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="80.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -801,11 +718,11 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="63" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -821,389 +738,233 @@
       <c r="I2" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="2" customFormat="1" ht="96" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3">
         <v>276.39320972463588</v>
       </c>
-      <c r="I3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J3" s="6" t="s">
+      <c r="I3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="80" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>15</v>
       </c>
       <c r="B4">
         <v>-387.88448976136772</v>
       </c>
-      <c r="D4">
-        <v>-387.88448976136772</v>
-      </c>
-      <c r="G4">
-        <v>-387.88448976136772</v>
-      </c>
       <c r="I4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J4" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>148.4099494288144</v>
+      </c>
+      <c r="I5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" s="2" customFormat="1" ht="64" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="B6">
+        <v>117.0310068038505</v>
+      </c>
+      <c r="I6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>17</v>
-      </c>
-      <c r="B5" s="2">
-        <v>148.4099494288144</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="2">
-        <v>117.0310068038505</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="64" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>21</v>
       </c>
       <c r="B7">
         <v>415.00617525975582</v>
       </c>
-      <c r="D7">
-        <v>415.00617525975582</v>
-      </c>
-      <c r="H7">
-        <v>415.00617525975582</v>
-      </c>
       <c r="I7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="64" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B8">
         <v>87.86865544914879</v>
       </c>
-      <c r="C8">
-        <v>87.86865544914879</v>
-      </c>
-      <c r="E8">
-        <v>87.86865544914879</v>
-      </c>
       <c r="I8" t="s">
-        <v>2</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="80" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B9">
         <v>503.95253613149163</v>
       </c>
-      <c r="C9">
-        <v>503.95253613149163</v>
-      </c>
-      <c r="E9">
-        <v>503.95253613149163</v>
-      </c>
       <c r="I9" t="s">
-        <v>2</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" s="2" customFormat="1" ht="80" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10">
         <v>269.90349136839302</v>
       </c>
-      <c r="I10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="80" x14ac:dyDescent="0.2">
+      <c r="I10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B11">
         <v>96.113815876822159</v>
       </c>
-      <c r="C11">
-        <v>96.113815876822159</v>
-      </c>
-      <c r="E11">
-        <v>96.113815876822159</v>
-      </c>
       <c r="I11" t="s">
-        <v>2</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="64" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="B12">
         <v>-151.4124688981552</v>
       </c>
-      <c r="D12">
-        <v>-151.4124688981552</v>
-      </c>
-      <c r="G12">
-        <v>-151.4124688981552</v>
-      </c>
       <c r="I12" t="s">
-        <v>3</v>
-      </c>
-      <c r="J12" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B13">
         <v>-189.26896537445259</v>
       </c>
-      <c r="C13">
-        <v>-189.26896537445259</v>
-      </c>
-      <c r="F13">
-        <v>-189.26896537445259</v>
-      </c>
       <c r="I13" t="s">
-        <v>2</v>
-      </c>
-      <c r="J13" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B14">
         <v>-202.9847143898794</v>
       </c>
-      <c r="C14">
-        <v>-202.9847143898794</v>
-      </c>
-      <c r="F14">
-        <v>-202.9847143898794</v>
-      </c>
       <c r="I14" t="s">
-        <v>2</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="B15">
         <v>-156.82028933312361</v>
       </c>
-      <c r="C15">
-        <v>-156.82028933312361</v>
-      </c>
-      <c r="F15">
-        <v>-156.82028933312361</v>
-      </c>
       <c r="I15" t="s">
-        <v>2</v>
-      </c>
-      <c r="J15" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="80" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="B16">
         <v>-111.53031497214729</v>
       </c>
-      <c r="C16">
-        <v>-111.53031497214729</v>
-      </c>
-      <c r="F16">
-        <v>-111.53031497214729</v>
-      </c>
       <c r="I16" t="s">
-        <v>2</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="B17">
         <v>-232.4417007363582</v>
       </c>
-      <c r="D17" s="3">
-        <v>-232.4417007363582</v>
-      </c>
-      <c r="G17">
-        <v>-232.4417007363582</v>
-      </c>
       <c r="I17" t="s">
-        <v>3</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="B18">
         <v>-249.5974496202042</v>
       </c>
-      <c r="D18">
-        <v>-249.5974496202042</v>
-      </c>
-      <c r="G18">
-        <v>-249.5974496202042</v>
-      </c>
       <c r="I18" t="s">
-        <v>3</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="B19">
         <v>-529.17092465149221</v>
       </c>
-      <c r="D19">
-        <v>-529.17092465149221</v>
-      </c>
-      <c r="G19">
-        <v>-529.17092465149221</v>
-      </c>
       <c r="I19" t="s">
-        <v>3</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="80" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B20">
         <v>-146.78116308087399</v>
       </c>
-      <c r="D20">
-        <v>-146.78116308087399</v>
-      </c>
-      <c r="G20">
-        <v>-146.78116308087399</v>
-      </c>
       <c r="I20" t="s">
-        <v>3</v>
-      </c>
-      <c r="J20" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="B21">
         <v>-148.2249838679231</v>
       </c>
-      <c r="D21">
-        <v>-148.2249838679231</v>
-      </c>
-      <c r="G21">
-        <v>-148.2249838679231</v>
-      </c>
       <c r="I21" t="s">
-        <v>3</v>
-      </c>
-      <c r="J21" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="B22">
         <v>-246.37821805298611</v>
       </c>
-      <c r="D22">
-        <v>-246.37821805298611</v>
-      </c>
-      <c r="G22">
-        <v>-246.37821805298611</v>
-      </c>
       <c r="I22" t="s">
-        <v>3</v>
-      </c>
-      <c r="J22" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="B23">
         <v>-87.722760721289646</v>
@@ -1211,13 +972,10 @@
       <c r="I23" t="s">
         <v>13</v>
       </c>
-      <c r="J23" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="B24">
         <v>-172.83179207606861</v>
@@ -1226,9 +984,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="B25">
         <v>-141.21637310006321</v>
@@ -1237,9 +995,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="B26">
         <v>-161.06960258571269</v>
@@ -1248,9 +1006,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="B27">
         <v>-202.57199864455171</v>
@@ -1259,9 +1017,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="B28">
         <v>-163.31804264167221</v>
@@ -1270,9 +1028,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="B29">
         <v>-152.92923732444689</v>
@@ -1281,9 +1039,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="B30">
         <v>-248.45256107553939</v>
@@ -1292,9 +1050,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="B31">
         <v>-1199.209304600121</v>
@@ -1303,9 +1061,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B32">
         <v>391.86138027946919</v>
@@ -1316,7 +1074,7 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="B33">
         <v>108.2317293907218</v>
@@ -1327,7 +1085,7 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="B34">
         <v>-261.5619937281686</v>
@@ -1338,7 +1096,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="B35">
         <v>-107.88515860470319</v>
@@ -1349,7 +1107,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="B36">
         <v>-182.8788031923161</v>
@@ -1360,7 +1118,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B37">
         <v>-183.42798776198691</v>
@@ -1371,7 +1129,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="B38">
         <v>-192.6147477522621</v>
@@ -1382,7 +1140,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="B39">
         <v>1748.3550672281619</v>
@@ -1393,7 +1151,7 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="B40">
         <v>-402.29826229755741</v>
@@ -1404,7 +1162,7 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="B41">
         <v>-138.6862505995087</v>
@@ -1415,7 +1173,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="B42">
         <v>-230.6493234163718</v>
@@ -1426,7 +1184,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="B43">
         <v>-1782.0190466026061</v>
@@ -1437,7 +1195,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="B44">
         <v>92.217497605615179</v>
@@ -1448,7 +1206,7 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="B45">
         <v>477.6407083384322</v>
@@ -1459,7 +1217,7 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="B46">
         <v>161.86215832132129</v>
@@ -1470,7 +1228,7 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="B47">
         <v>-273.05665714327893</v>
@@ -1481,7 +1239,7 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="B48">
         <v>146.1973513648887</v>
@@ -1492,7 +1250,7 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="B49">
         <v>114.64160770773699</v>
@@ -1503,7 +1261,7 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="B50">
         <v>133.22528008284601</v>
@@ -1514,7 +1272,7 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="B51">
         <v>-203.91844288041531</v>
@@ -1525,7 +1283,7 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="B52">
         <v>-446.16251606515442</v>
@@ -1536,7 +1294,7 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="B53">
         <v>93.513879965796519</v>
@@ -1547,7 +1305,7 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="B54">
         <v>-192.33581616385399</v>
@@ -1558,7 +1316,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="B55">
         <v>-176.92371282897821</v>
@@ -1569,7 +1327,7 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="B56">
         <v>-207.28690503464159</v>
@@ -1580,7 +1338,7 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="B57">
         <v>-165.0011653349533</v>
@@ -1591,7 +1349,7 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="B58">
         <v>-276.38945753885929</v>
@@ -1602,7 +1360,7 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="B59">
         <v>-120.1009540721557</v>
@@ -1613,7 +1371,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="B60">
         <v>-143.1113566126474</v>
@@ -1624,7 +1382,7 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="B61">
         <v>-428.79182457489537</v>
@@ -1635,7 +1393,7 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="B62">
         <v>-657.44251936497039</v>
@@ -1646,7 +1404,7 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="B63">
         <v>-2041.780924862881</v>
@@ -1657,7 +1415,7 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="B64">
         <v>615.86628034078262</v>
@@ -1668,7 +1426,7 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="B65">
         <v>-169.59377942450891</v>
@@ -1679,7 +1437,7 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="B66">
         <v>-89.290345938567185</v>
@@ -1690,7 +1448,7 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="B67">
         <v>-984.66883793782119</v>
@@ -1701,7 +1459,7 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="B68">
         <v>-476.00040837070628</v>
@@ -1712,7 +1470,7 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="B69">
         <v>179.54472327198059</v>
@@ -1723,7 +1481,7 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="B70">
         <v>166.5617790268318</v>
@@ -1734,7 +1492,7 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="B71">
         <v>-180.10847121243651</v>
@@ -1745,7 +1503,7 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="B72">
         <v>-179.83145417219279</v>
@@ -1756,7 +1514,7 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="B73">
         <v>-552.22911894411504</v>
@@ -1767,7 +1525,7 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="B74">
         <v>-234.61385357430859</v>
@@ -1778,7 +1536,7 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>106</v>
+        <v>85</v>
       </c>
       <c r="B75">
         <v>202.46136313468651</v>
@@ -1789,7 +1547,7 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="B76">
         <v>-106.5970450688274</v>
@@ -1800,7 +1558,7 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="B77">
         <v>-1051.6635574296449</v>
@@ -1811,7 +1569,7 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="B78">
         <v>-540.46550103801428</v>
@@ -1822,7 +1580,7 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="B79">
         <v>-197.7441439976659</v>
@@ -1833,7 +1591,7 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="B80">
         <v>-700.94624941174834</v>
@@ -1844,7 +1602,7 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>112</v>
+        <v>91</v>
       </c>
       <c r="B81">
         <v>-412.80577790767512</v>
@@ -1855,7 +1613,7 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="B82">
         <v>-640.16266533291071</v>
@@ -1866,7 +1624,7 @@
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="B83">
         <v>-515.37490113762385</v>
@@ -1877,7 +1635,7 @@
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="B84">
         <v>-214.08815960384689</v>
@@ -1888,7 +1646,7 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>116</v>
+        <v>95</v>
       </c>
       <c r="B85">
         <v>844.14424346889075</v>
@@ -1899,7 +1657,7 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="B86">
         <v>-377.90035722856311</v>
@@ -1910,7 +1668,7 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="B87">
         <v>-200.3390287029126</v>
@@ -1921,7 +1679,7 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="B88">
         <v>-236.26023728124079</v>

</xml_diff>

<commit_message>
Also this promt works not as what I would want, I'll change it back to the original versione
</commit_message>
<xml_diff>
--- a/FISCAL/Fiscal_LDC/Classified_Fiscal_Events_Top5Percent.xlsx
+++ b/FISCAL/Fiscal_LDC/Classified_Fiscal_Events_Top5Percent.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzodelcol/Desktop/GIT/RA_4_Caggiano/FISCAL/Fiscal_LDC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DECA611-1D79-1140-82BC-1908DBCBC7B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{174639B1-7540-6344-98C9-30ACD6ACA484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4400" yWindow="-21600" windowWidth="16360" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20320" yWindow="0" windowWidth="20320" windowHeight="14920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="120">
   <si>
     <t>date</t>
   </si>
@@ -55,75 +55,132 @@
     <t>1961-03-27</t>
   </si>
   <si>
-    <t>The House of Representatives approved the Area Redevelopment Act (H.R. 4569) on March 28, 1961, authorizing significant federal funds for loans and grants to economically distressed areas. This legislative action represents a direct increase in government spending.</t>
+    <t>The massive fiscal shock on 1961-03-27 is primarily driven by the widespread reporting and analysis of President Kennedy's comprehensive economic message sent to Congress on March 24, 1961. This message outlined a broad array of significant government spending proposals aimed at stimulating the economy and addressing social needs. Key spending initiatives included the extension of unemployment benefits, increased aid to depressed areas, new housing programs, accelerated highway construction, and a boost in defense spending. While the message also proposed tax changes (e.g., an investment tax credit), the sheer volume and breadth of these direct government outlays represent the dominant factor for a peak daily fiscal shock at this time.</t>
   </si>
   <si>
     <t>1976-11-15</t>
   </si>
   <si>
+    <t>1980-11-06</t>
+  </si>
+  <si>
+    <t>The massive fiscal shock on 1980-11-06 is primarily driven by the outcome of the 1980 Presidential Election on November 4th. Ronald Reagan's landslide victory, confirmed and widely reported on November 5th and 6th, signaled a dramatic shift in economic policy towards 'Reaganomics.' A cornerstone of Reagan's platform was significant tax cuts, which were subsequently enacted as the Economic Recovery Tax Act of 1981 (ERTA). The market's immediate reaction to the election results reflected the strong expectation of these major tax reductions, making tax changes the dominant fiscal policy driver.</t>
+  </si>
+  <si>
+    <t>1981-02-18</t>
+  </si>
+  <si>
+    <t>On February 18, 1981, President Ronald Reagan delivered his 'Program for Economic Recovery' speech to a joint session of Congress. This comprehensive plan outlined significant cuts in federal spending and a major proposal for a 30% across-the-board cut in individual income tax rates over three years (the Kemp-Roth tax cut). While the plan included both spending cuts (G) and tax cuts (T), the proposed tax reductions were a cornerstone of Reagan's supply-side economic philosophy and represented a massive, defining shift in fiscal policy, making them the most dominant factor in the macroeconomic news cycle and the primary driver of the fiscal shock on this date.</t>
+  </si>
+  <si>
+    <t>1993-02-15</t>
+  </si>
+  <si>
+    <t>The massive fiscal shock on 1993-02-15 was primarily driven by the widely reported and leaked details of President Clinton's comprehensive economic plan, which was formally unveiled on February 17, 1993. In the 48-to-72-hour window around this date, news outlets extensively covered the plan's components, with a significant focus on proposed tax increases. These included raising the top marginal income tax rates for individuals and corporations, increasing the taxation of Social Security benefits for higher earners, and introducing a new energy (BTU) tax. While the plan also included spending cuts, the substantial and broad-reaching tax increases were a dominant and highly discussed feature, likely triggering the outsized macroeconomic reaction.</t>
+  </si>
+  <si>
+    <t>1993-08-09</t>
+  </si>
+  <si>
+    <t>The massive fiscal shock on 1993-08-09 is primarily driven by the final legislative actions surrounding the Omnibus Budget Reconciliation Act of 1993 (OBRA-93). The bill passed the House on August 5th and the Senate on August 6th, and was signed into law by President Clinton on August 10th. While OBRA-93 was a comprehensive deficit reduction package that included both significant tax increases and spending cuts, the spending reductions, totaling approximately $255 billion over five years (including cuts to Medicare, defense, and other discretionary programs), were slightly larger in magnitude than the tax increases ($241 billion). Therefore, Government Spending (G) is identified as the dominant factor.</t>
+  </si>
+  <si>
+    <t>1995-10-20</t>
+  </si>
+  <si>
+    <t>The fiscal shock on 1995-10-20 was primarily driven by the intense budget negotiations between the Republican-controlled Congress and President Clinton. Around this date, the House of Representatives was advancing or had just passed its comprehensive budget reconciliation bill, which included massive proposed cuts to federal spending, particularly Medicare, Medicaid, and welfare programs, as part of a plan to balance the budget in seven years. This legislative action, focused on reducing government outlays, represented a significant fiscal shock related to government spending.</t>
+  </si>
+  <si>
+    <t>1995-11-20</t>
+  </si>
+  <si>
+    <t>The massive fiscal shock on 1995-11-20 was primarily driven by Government Spending (G). This date marks the reopening of the federal government after its first shutdown (November 13-19, 1995) due to a budget impasse between President Clinton and the Republican-controlled Congress. The immediate shock on this day was the resumption of government operations and services, which are direct components of government spending. While the broader budget negotiations involved both proposed spending cuts and tax cuts, the shutdown itself and its temporary resolution were fundamentally about the authorization and appropriation of federal spending.</t>
+  </si>
+  <si>
+    <t>1997-09-03</t>
+  </si>
+  <si>
+    <t>The 'massive, peak daily fiscal shock' on 1997-09-03 was primarily driven by the ongoing public and financial community's assimilation and detailed analysis of the Taxpayer Relief Act of 1997. Signed into law on August 5, 1997, this act introduced significant tax cuts, including the child tax credit, education tax credits, and capital gains tax reductions. In the 48-to-72-hour window around September 3rd, news cycles were heavily focused on explaining the complexities and broad implications of these tax changes for individuals and businesses, leading to a clearer understanding of the substantial impact on federal revenues and the economy. This widespread realization of the scale and specifics of the tax cuts likely triggered the recorded fiscal shock.</t>
+  </si>
+  <si>
+    <t>2000-01-26</t>
+  </si>
+  <si>
+    <t>The massive fiscal shock on or around January 26, 2000, is primarily attributable to President Clinton's State of the Union address delivered on January 27, 2000. This address outlined a comprehensive plan for allocating the projected budget surplus, emphasizing significant new government spending and commitments to existing entitlement programs like Social Security and Medicare, alongside substantial debt reduction. While targeted tax cuts were also proposed, the dominant fiscal policy news centered on the magnitude of these proposed allocations and new spending initiatives, rather than revenue changes.</t>
+  </si>
+  <si>
+    <t>2001-01-26</t>
+  </si>
+  <si>
+    <t>The fiscal shock on 2001-01-26 was primarily driven by intense news and political activity surrounding newly inaugurated President George W. Bush's push for his signature tax cut plan. In the days immediately following his inauguration (January 20th), Bush met with congressional leaders and publicly advocated for a substantial, multi-trillion-dollar tax reduction over the next decade. This high-profile initiative, a core promise of his campaign, dominated the fiscal policy news cycle and represented a significant anticipated change in government revenue, thus classifying it as a Tax change (T).</t>
+  </si>
+  <si>
+    <t>2001-09-12</t>
+  </si>
+  <si>
+    <t>The 9/11 terrorist attacks on September 11, 2001, triggered an immediate and massive government response. This included emergency appropriations for rescue, recovery, and national security, leading to a significant, sudden increase in government spending. The announcement and legislative efforts for a $40 billion emergency supplemental appropriation began immediately after the attacks, representing a peak daily fiscal shock driven by government expenditure.</t>
+  </si>
+  <si>
+    <t>2001-10-01</t>
+  </si>
+  <si>
+    <t>The fiscal shock on 2001-10-01 is primarily driven by the start of the new fiscal year (FY2002) and the immediate, massive increase in government spending for national security, defense, and homeland security in the wake of the September 11th attacks. While emergency appropriations (like the $40 billion supplemental) were passed earlier in September, October 1st marked the official commencement of the new fiscal year, solidifying the implementation and anticipation of significant government outlays for the 'War on Terror' and domestic security enhancements. News in this window would have been dominated by the impending military response and the associated, unprecedented spending commitments.</t>
+  </si>
+  <si>
+    <t>2002-01-24</t>
+  </si>
+  <si>
+    <t>On January 24, 2002, the U.S. House of Representatives passed the 'Job Creation and Worker Assistance Act of 2002' (H.R. 3090). This significant economic stimulus package was primarily driven by tax changes, including provisions for 30% bonus depreciation for businesses and other tax relief measures, aimed at stimulating the economy following the 2001 recession and the 9/11 attacks. While it also included extended unemployment benefits, the dominant fiscal policy news and the largest component of the shock were the business tax cuts.</t>
+  </si>
+  <si>
+    <t>2002-05-13</t>
+  </si>
+  <si>
+    <t>On May 13, 2002, President George W. Bush signed the Farm Security and Rural Investment Act of 2002 (the 2002 Farm Bill) into law. This comprehensive legislation significantly increased government spending on agricultural subsidies and conservation programs over the next decade, representing a substantial fiscal commitment primarily driven by Government Spending (G).</t>
+  </si>
+  <si>
+    <t>2002-12-09</t>
+  </si>
+  <si>
+    <t>The news cycle around 2002-12-09 was dominated by reports detailing the Bush administration's preparations for a significant new economic stimulus package. These reports, widely covered in major news outlets, emphasized that the core of the proposed package would be substantial tax cuts, including accelerating existing tax reductions and potentially new measures like dividend tax relief, aimed at boosting the sluggish economy. This intense focus on an impending large-scale tax reduction plan would constitute a major fiscal shock.</t>
+  </si>
+  <si>
+    <t>2003-01-06</t>
+  </si>
+  <si>
+    <t>The fiscal shock on or around January 6, 2003, was primarily driven by the anticipation and subsequent unveiling of President George W. Bush's economic stimulus package. Formally announced on January 7th, but widely discussed and leaked in the preceding days, this package was heavily centered on significant tax cuts, including the elimination of the tax on stock dividends, acceleration of income tax rate reductions, and making previous tax cuts permanent, aiming to stimulate the economy.</t>
+  </si>
+  <si>
+    <t>2003-02-03</t>
+  </si>
+  <si>
+    <t>On February 3, 2003, President George W. Bush released his FY2004 budget proposal. A central and highly publicized component of this budget was a significant package of proposed tax cuts, most notably the elimination of taxes on corporate dividends. This new tax policy initiative, alongside proposals to make the 2001 tax cuts permanent and accelerate other provisions, represented a major fiscal policy announcement aimed at stimulating the economy and was a dominant feature of the news cycle, triggering a substantial macroeconomic reaction related to changes in revenue policy.</t>
+  </si>
+  <si>
+    <t>2003-07-16</t>
+  </si>
+  <si>
+    <t>On July 16, 2003, the U.S. House of Representatives passed the FY2004 Defense Appropriations bill (H.R. 2658) by a vote of 399-19. This legislative action authorized significant government spending for military operations and defense, representing a major fiscal policy event related to government outlays.</t>
+  </si>
+  <si>
+    <t>2003-08-26</t>
+  </si>
+  <si>
+    <t>In the days surrounding August 26, 2003, news was breaking that the Bush administration was preparing to request a massive supplemental appropriation for military operations and reconstruction efforts in Iraq and Afghanistan. While the formal request for $87 billion was made on September 2, 2003, the anticipation and imminent announcement of such a substantial increase in federal outlays for defense and foreign aid constituted a major fiscal shock related to government spending (G) in the preceding days.</t>
+  </si>
+  <si>
+    <t>2003-08-27</t>
+  </si>
+  <si>
+    <t>The Congressional Budget Office (CBO) released its 'Budget and Economic Outlook: An Update' on August 26, 2003. This report projected a record federal budget deficit of $401 billion for FY2003, a significant upward revision from previous estimates. News coverage around August 27, 2003, widely attributed this massive increase in the deficit projection primarily to the revenue losses from the Jobs and Growth Tax Relief Reconciliation Act of 2003 (JGTRRA), which had been enacted in May and included substantial tax cuts on dividends, capital gains, and income. While increased spending for defense and homeland security also contributed, the CBO's quantification of the impact of these recent, large-scale tax changes was a dominant factor in the fiscal shock.</t>
+  </si>
+  <si>
+    <t>2004-10-07</t>
+  </si>
+  <si>
     <t>N</t>
   </si>
   <si>
-    <t>1980-11-06</t>
-  </si>
-  <si>
-    <t>1981-02-18</t>
-  </si>
-  <si>
-    <t>1993-02-15</t>
-  </si>
-  <si>
-    <t>1993-08-09</t>
-  </si>
-  <si>
-    <t>1995-10-20</t>
-  </si>
-  <si>
-    <t>1995-11-20</t>
-  </si>
-  <si>
-    <t>1997-09-03</t>
-  </si>
-  <si>
-    <t>2000-01-26</t>
-  </si>
-  <si>
-    <t>2001-01-26</t>
-  </si>
-  <si>
-    <t>2001-09-12</t>
-  </si>
-  <si>
-    <t>2001-10-01</t>
-  </si>
-  <si>
-    <t>2002-01-24</t>
-  </si>
-  <si>
-    <t>2002-05-13</t>
-  </si>
-  <si>
-    <t>2002-12-09</t>
-  </si>
-  <si>
-    <t>2003-01-06</t>
-  </si>
-  <si>
-    <t>2003-02-03</t>
-  </si>
-  <si>
-    <t>2003-07-16</t>
-  </si>
-  <si>
-    <t>2003-08-26</t>
-  </si>
-  <si>
-    <t>2003-08-27</t>
-  </si>
-  <si>
-    <t>2004-10-07</t>
-  </si>
-  <si>
     <t>2004-11-04</t>
   </si>
   <si>
@@ -317,13 +374,39 @@
   </si>
   <si>
     <t>2025-07-03</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The massive fiscal shock on 1976-11-15 is primarily driven by news surrounding the incoming Carter administration's plans for a significant economic stimulus package. Following the November 2nd election, President-elect Jimmy Carter's economic transition team began actively discussing and signaling a strong commitment to combating high unemployment. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Corpo)"/>
+      </rPr>
+      <t>While tax cuts were part of the discussion, the dominant factor in the news cycle around this date was the strong emphasis on direct government spending for job creation programs and public works.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> This focus on active government intervention to stimulate employment, a key promise of Carter's campaign, signaled a substantial increase in government outlays, leading to a significant fiscal shock.</t>
+    </r>
+  </si>
+  <si>
+    <t>Secondo me è TAX shock, Negative Tax Shock --&gt; decrease in Taxes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -335,15 +418,25 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri (Corpo)"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -373,13 +466,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -683,14 +783,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:K88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="80.5" customWidth="1"/>
+    <col min="10" max="10" width="87.33203125" style="3" customWidth="1"/>
+    <col min="11" max="11" width="52" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -718,11 +820,11 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -738,954 +840,1137 @@
       <c r="I2" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="3" spans="1:11" s="4" customFormat="1" ht="128" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="4">
         <v>276.39320972463588</v>
       </c>
-      <c r="I3" t="s">
+      <c r="C3" s="4">
+        <v>276.39320972463588</v>
+      </c>
+      <c r="E3" s="4">
+        <v>276.39320972463588</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="96" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>14</v>
       </c>
       <c r="B4">
         <v>-387.88448976136772</v>
       </c>
+      <c r="D4">
+        <v>-387.88448976136772</v>
+      </c>
+      <c r="G4">
+        <v>-387.88448976136772</v>
+      </c>
       <c r="I4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>15</v>
       </c>
       <c r="B5">
         <v>148.4099494288144</v>
       </c>
+      <c r="D5">
+        <v>148.4099494288144</v>
+      </c>
+      <c r="H5">
+        <v>148.4099494288144</v>
+      </c>
       <c r="I5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6">
         <v>117.0310068038505</v>
       </c>
+      <c r="D6">
+        <v>117.0310068038505</v>
+      </c>
+      <c r="H6">
+        <v>117.0310068038505</v>
+      </c>
       <c r="I6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B7">
         <v>415.00617525975582</v>
       </c>
+      <c r="C7">
+        <v>415.00617525975582</v>
+      </c>
+      <c r="E7">
+        <v>415.00617525975582</v>
+      </c>
       <c r="I7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B8">
         <v>87.86865544914879</v>
       </c>
+      <c r="C8">
+        <v>87.86865544914879</v>
+      </c>
+      <c r="E8">
+        <v>87.86865544914879</v>
+      </c>
       <c r="I8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B9">
         <v>503.95253613149163</v>
       </c>
+      <c r="C9">
+        <v>503.95253613149163</v>
+      </c>
+      <c r="E9">
+        <v>503.95253613149163</v>
+      </c>
       <c r="I9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B10">
         <v>269.90349136839302</v>
       </c>
+      <c r="D10">
+        <v>269.90349136839302</v>
+      </c>
+      <c r="H10">
+        <v>269.90349136839302</v>
+      </c>
       <c r="I10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B11">
         <v>96.113815876822159</v>
       </c>
+      <c r="C11">
+        <v>96.113815876822159</v>
+      </c>
+      <c r="E11">
+        <v>96.113815876822159</v>
+      </c>
       <c r="I11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="B12">
         <v>-151.4124688981552</v>
       </c>
+      <c r="D12">
+        <v>-151.4124688981552</v>
+      </c>
+      <c r="G12">
+        <v>-151.4124688981552</v>
+      </c>
       <c r="I12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B13">
         <v>-189.26896537445259</v>
       </c>
+      <c r="C13">
+        <v>-189.26896537445259</v>
+      </c>
+      <c r="F13">
+        <v>-189.26896537445259</v>
+      </c>
       <c r="I13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="B14">
         <v>-202.9847143898794</v>
       </c>
+      <c r="C14">
+        <v>-202.9847143898794</v>
+      </c>
+      <c r="F14">
+        <v>-202.9847143898794</v>
+      </c>
       <c r="I14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B15">
         <v>-156.82028933312361</v>
       </c>
+      <c r="D15">
+        <v>-156.82028933312361</v>
+      </c>
+      <c r="G15">
+        <v>-156.82028933312361</v>
+      </c>
       <c r="I15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B16">
         <v>-111.53031497214729</v>
       </c>
+      <c r="C16">
+        <v>-111.53031497214729</v>
+      </c>
+      <c r="F16">
+        <v>-111.53031497214729</v>
+      </c>
       <c r="I16" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="B17">
         <v>-232.4417007363582</v>
       </c>
+      <c r="D17">
+        <v>-232.4417007363582</v>
+      </c>
+      <c r="G17">
+        <v>-232.4417007363582</v>
+      </c>
       <c r="I17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="B18">
         <v>-249.5974496202042</v>
       </c>
+      <c r="D18">
+        <v>-249.5974496202042</v>
+      </c>
+      <c r="G18">
+        <v>-249.5974496202042</v>
+      </c>
       <c r="I18" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="96" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="B19">
         <v>-529.17092465149221</v>
       </c>
+      <c r="D19">
+        <v>-529.17092465149221</v>
+      </c>
+      <c r="G19">
+        <v>-529.17092465149221</v>
+      </c>
       <c r="I19" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" s="4" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="4">
         <v>-146.78116308087399</v>
       </c>
-      <c r="I20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C20" s="4">
+        <v>-146.78116308087399</v>
+      </c>
+      <c r="F20" s="4">
+        <v>-146.78116308087399</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="B21">
         <v>-148.2249838679231</v>
       </c>
+      <c r="C21">
+        <v>-148.2249838679231</v>
+      </c>
+      <c r="F21">
+        <v>-148.2249838679231</v>
+      </c>
       <c r="I21" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" s="4" customFormat="1" ht="128" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="4">
         <v>-246.37821805298611</v>
       </c>
-      <c r="I22" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="D22" s="4">
+        <v>-246.37821805298611</v>
+      </c>
+      <c r="G22" s="4">
+        <v>-246.37821805298611</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B23">
         <v>-87.722760721289646</v>
       </c>
       <c r="I23" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="B24">
         <v>-172.83179207606861</v>
       </c>
       <c r="I24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="B25">
         <v>-141.21637310006321</v>
       </c>
       <c r="I25" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="B26">
         <v>-161.06960258571269</v>
       </c>
       <c r="I26" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="B27">
         <v>-202.57199864455171</v>
       </c>
       <c r="I27" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="B28">
         <v>-163.31804264167221</v>
       </c>
       <c r="I28" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="B29">
         <v>-152.92923732444689</v>
       </c>
       <c r="I29" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="B30">
         <v>-248.45256107553939</v>
       </c>
       <c r="I30" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="B31">
         <v>-1199.209304600121</v>
       </c>
       <c r="I31" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="B32">
         <v>391.86138027946919</v>
       </c>
       <c r="I32" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="B33">
         <v>108.2317293907218</v>
       </c>
       <c r="I33" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="B34">
         <v>-261.5619937281686</v>
       </c>
       <c r="I34" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="B35">
         <v>-107.88515860470319</v>
       </c>
       <c r="I35" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="B36">
         <v>-182.8788031923161</v>
       </c>
       <c r="I36" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="B37">
         <v>-183.42798776198691</v>
       </c>
       <c r="I37" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="B38">
         <v>-192.6147477522621</v>
       </c>
       <c r="I38" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="B39">
         <v>1748.3550672281619</v>
       </c>
       <c r="I39" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="B40">
         <v>-402.29826229755741</v>
       </c>
       <c r="I40" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="B41">
         <v>-138.6862505995087</v>
       </c>
       <c r="I41" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="B42">
         <v>-230.6493234163718</v>
       </c>
       <c r="I42" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="B43">
         <v>-1782.0190466026061</v>
       </c>
       <c r="I43" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="B44">
         <v>92.217497605615179</v>
       </c>
       <c r="I44" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="B45">
         <v>477.6407083384322</v>
       </c>
       <c r="I45" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="B46">
         <v>161.86215832132129</v>
       </c>
       <c r="I46" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="B47">
         <v>-273.05665714327893</v>
       </c>
       <c r="I47" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="B48">
         <v>146.1973513648887</v>
       </c>
       <c r="I48" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="B49">
         <v>114.64160770773699</v>
       </c>
       <c r="I49" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="B50">
         <v>133.22528008284601</v>
       </c>
       <c r="I50" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="B51">
         <v>-203.91844288041531</v>
       </c>
       <c r="I51" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="B52">
         <v>-446.16251606515442</v>
       </c>
       <c r="I52" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="B53">
         <v>93.513879965796519</v>
       </c>
       <c r="I53" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="B54">
         <v>-192.33581616385399</v>
       </c>
       <c r="I54" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="B55">
         <v>-176.92371282897821</v>
       </c>
       <c r="I55" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="B56">
         <v>-207.28690503464159</v>
       </c>
       <c r="I56" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="B57">
         <v>-165.0011653349533</v>
       </c>
       <c r="I57" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="B58">
         <v>-276.38945753885929</v>
       </c>
       <c r="I58" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="B59">
         <v>-120.1009540721557</v>
       </c>
       <c r="I59" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B60">
         <v>-143.1113566126474</v>
       </c>
       <c r="I60" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="B61">
         <v>-428.79182457489537</v>
       </c>
       <c r="I61" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="B62">
         <v>-657.44251936497039</v>
       </c>
       <c r="I62" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="B63">
         <v>-2041.780924862881</v>
       </c>
       <c r="I63" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="B64">
         <v>615.86628034078262</v>
       </c>
       <c r="I64" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="B65">
         <v>-169.59377942450891</v>
       </c>
       <c r="I65" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="B66">
         <v>-89.290345938567185</v>
       </c>
       <c r="I66" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="B67">
         <v>-984.66883793782119</v>
       </c>
       <c r="I67" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="B68">
         <v>-476.00040837070628</v>
       </c>
       <c r="I68" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B69">
         <v>179.54472327198059</v>
       </c>
       <c r="I69" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="B70">
         <v>166.5617790268318</v>
       </c>
       <c r="I70" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="B71">
         <v>-180.10847121243651</v>
       </c>
       <c r="I71" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="B72">
         <v>-179.83145417219279</v>
       </c>
       <c r="I72" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="B73">
         <v>-552.22911894411504</v>
       </c>
       <c r="I73" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="B74">
         <v>-234.61385357430859</v>
       </c>
       <c r="I74" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="B75">
         <v>202.46136313468651</v>
       </c>
       <c r="I75" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="B76">
         <v>-106.5970450688274</v>
       </c>
       <c r="I76" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="B77">
         <v>-1051.6635574296449</v>
       </c>
       <c r="I77" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="B78">
         <v>-540.46550103801428</v>
       </c>
       <c r="I78" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="B79">
         <v>-197.7441439976659</v>
       </c>
       <c r="I79" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="B80">
         <v>-700.94624941174834</v>
       </c>
       <c r="I80" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="B81">
         <v>-412.80577790767512</v>
       </c>
       <c r="I81" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
       <c r="B82">
         <v>-640.16266533291071</v>
       </c>
       <c r="I82" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
       <c r="B83">
         <v>-515.37490113762385</v>
       </c>
       <c r="I83" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="B84">
         <v>-214.08815960384689</v>
       </c>
       <c r="I84" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>95</v>
+        <v>114</v>
       </c>
       <c r="B85">
         <v>844.14424346889075</v>
       </c>
       <c r="I85" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="B86">
         <v>-377.90035722856311</v>
       </c>
       <c r="I86" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="B87">
         <v>-200.3390287029126</v>
       </c>
       <c r="I87" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="B88">
         <v>-236.26023728124079</v>
       </c>
       <c r="I88" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>